<commit_message>
chore: expand sample xlsx to 111 reviews
</commit_message>
<xml_diff>
--- a/public/samples/feedfocus-sample-reviews.xlsx
+++ b/public/samples/feedfocus-sample-reviews.xlsx
@@ -398,9 +398,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E112"/>
   <cols>
-    <col min="1" max="1" width="70.83203125" customWidth="1"/>
+    <col min="1" max="1" width="90.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
@@ -426,16 +426,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Приложение долго открывается (10–15 секунд).</v>
+        <v>Приложение долго открывается: 6 секунд до главного экрана. Особенно заметно утром.</v>
       </c>
       <c r="B2" t="str">
         <v>App Store</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-03-10</v>
+        <v>2026-03-11</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" t="str">
         <v>performance</v>
@@ -443,13 +443,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Поддержка отвечает через сутки, это слишком долго.</v>
+        <v>Поддержка отвечает слишком долго — ждал(а) 9 часов.</v>
       </c>
       <c r="B3" t="str">
-        <v>Support</v>
+        <v>Google Play</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-03-09</v>
+        <v>2026-03-10</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -460,16 +460,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Не могу найти, где изменить тариф. Навигация неочевидная.</v>
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
       </c>
       <c r="B4" t="str">
-        <v>Chat</v>
+        <v>Support</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-03-08</v>
+        <v>2026-03-09</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="str">
         <v>ux</v>
@@ -477,16 +477,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>После обновления приложение стало тормозить. Иногда зависает на главном экране.</v>
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
       </c>
       <c r="B5" t="str">
-        <v>Google Play</v>
+        <v>Chat</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-03-07</v>
+        <v>2026-03-08</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="str">
         <v>bug</v>
@@ -494,13 +494,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Слишком много шагов при регистрации. Хочется быстрее начать пользоваться.</v>
+        <v>Регистрация слишком сложная: 8 шагов — хочется меньше.</v>
       </c>
       <c r="B6" t="str">
-        <v>App Store</v>
+        <v>Form</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-03-06</v>
+        <v>2026-03-07</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -511,16 +511,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Оплата не прошла, но деньги списались. Пришлось писать в поддержку.</v>
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
       </c>
       <c r="B7" t="str">
-        <v>Support</v>
+        <v>App Store</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-03-05</v>
+        <v>2026-03-06</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="str">
         <v>billing</v>
@@ -528,16 +528,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Иногда при входе пишет «что-то пошло не так», без объяснения.</v>
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
       </c>
       <c r="B8" t="str">
-        <v>Chat</v>
+        <v>Google Play</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-03-04</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="str">
         <v>errors</v>
@@ -545,13 +545,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Пуш-уведомления приходят с задержкой. Бывает, что вовсе не приходят.</v>
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
       </c>
       <c r="B9" t="str">
-        <v>App Store</v>
+        <v>Support</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-03-03</v>
+        <v>2026-03-04</v>
       </c>
       <c r="D9">
         <v>3</v>
@@ -562,16 +562,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Хочу экспортировать данные, но не вижу кнопки экспорта.</v>
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
       </c>
       <c r="B10" t="str">
-        <v>Form</v>
+        <v>Chat</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-03-02</v>
+        <v>2026-03-03</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" t="str">
         <v>feature</v>
@@ -579,38 +579,1755 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>В целом ок, но интерфейс перегружен. Новичку сложно разобраться.</v>
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
       </c>
       <c r="B11" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2026-03-02</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Приложение долго открывается: 16 секунд до главного экрана.</v>
+      </c>
+      <c r="B12" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 19 часов.</v>
+      </c>
+      <c r="B13" t="str">
         <v>Google Play</v>
       </c>
-      <c r="C11" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="D11">
-        <v>3</v>
-      </c>
-      <c r="E11" t="str">
+      <c r="C13" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Интерфейс перегружен: Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2026-02-27</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14" t="str">
         <v>ux</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2026-02-26</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Регистрация слишком сложная: 4 шагов — хочется меньше.</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2026-02-25</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B17" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2026-02-24</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C18" t="str">
+        <v>2026-02-23</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C19" t="str">
+        <v>2026-02-22</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="E19" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C20" t="str">
+        <v>2026-02-21</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C21" t="str">
+        <v>2026-02-20</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Приложение долго открывается: 14 секунд до главного экрана. Особенно заметно утром.</v>
+      </c>
+      <c r="B22" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C22" t="str">
+        <v>2026-02-19</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+      <c r="E22" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 29 часов.</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C23" t="str">
+        <v>2026-02-18</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C24" t="str">
+        <v>2026-02-17</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+      <c r="E24" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C25" t="str">
+        <v>2026-02-16</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Регистрация слишком сложная: 7 шагов — хочется меньше.</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2026-02-15</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B27" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C27" t="str">
+        <v>2026-02-14</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C28" t="str">
+        <v>2026-02-13</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2026-02-12</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C30" t="str">
+        <v>2026-02-11</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C31" t="str">
+        <v>2026-02-10</v>
+      </c>
+      <c r="D31">
+        <v>4</v>
+      </c>
+      <c r="E31" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Приложение долго открывается: 12 секунд до главного экрана.</v>
+      </c>
+      <c r="B32" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C32" t="str">
+        <v>2026-02-09</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 39 часов.</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="E33" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C34" t="str">
+        <v>2026-02-07</v>
+      </c>
+      <c r="D34">
+        <v>4</v>
+      </c>
+      <c r="E34" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2026-02-06</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Регистрация слишком сложная: 10 шагов — хочется меньше.</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C36" t="str">
+        <v>2026-02-05</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B37" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2026-02-04</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2026-02-03</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C39" t="str">
+        <v>2026-02-02</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C40" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="D40">
+        <v>4</v>
+      </c>
+      <c r="E40" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C41" t="str">
+        <v>2026-01-31</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Приложение долго открывается: 10 секунд до главного экрана. Особенно заметно утром.</v>
+      </c>
+      <c r="B42" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2026-01-30</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 9 часов.</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C43" t="str">
+        <v>2026-01-29</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Интерфейс перегружен: Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2026-01-28</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+      <c r="E44" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C45" t="str">
+        <v>2026-01-27</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Регистрация слишком сложная: 6 шагов — хочется меньше.</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C46" t="str">
+        <v>2026-01-26</v>
+      </c>
+      <c r="D46">
+        <v>3</v>
+      </c>
+      <c r="E46" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B47" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C47" t="str">
+        <v>2026-01-25</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C48" t="str">
+        <v>2026-01-24</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C49" t="str">
+        <v>2026-01-23</v>
+      </c>
+      <c r="D49">
+        <v>4</v>
+      </c>
+      <c r="E49" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C50" t="str">
+        <v>2026-01-22</v>
+      </c>
+      <c r="D50">
+        <v>2</v>
+      </c>
+      <c r="E50" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C51" t="str">
+        <v>2026-01-21</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Приложение долго открывается: 8 секунд до главного экрана.</v>
+      </c>
+      <c r="B52" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C52" t="str">
+        <v>2026-01-20</v>
+      </c>
+      <c r="D52">
+        <v>3</v>
+      </c>
+      <c r="E52" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 19 часов.</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C53" t="str">
+        <v>2026-01-19</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C54" t="str">
+        <v>2026-01-18</v>
+      </c>
+      <c r="D54">
+        <v>3</v>
+      </c>
+      <c r="E54" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C55" t="str">
+        <v>2026-01-17</v>
+      </c>
+      <c r="D55">
+        <v>3</v>
+      </c>
+      <c r="E55" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Регистрация слишком сложная: 9 шагов — хочется меньше.</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C56" t="str">
+        <v>2026-01-16</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="E56" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B57" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C57" t="str">
+        <v>2026-01-15</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C58" t="str">
+        <v>2026-01-14</v>
+      </c>
+      <c r="D58">
+        <v>3</v>
+      </c>
+      <c r="E58" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C59" t="str">
+        <v>2026-01-13</v>
+      </c>
+      <c r="D59">
+        <v>2</v>
+      </c>
+      <c r="E59" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C60" t="str">
+        <v>2026-01-12</v>
+      </c>
+      <c r="D60">
+        <v>3</v>
+      </c>
+      <c r="E60" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C61" t="str">
+        <v>2026-01-11</v>
+      </c>
+      <c r="D61">
+        <v>4</v>
+      </c>
+      <c r="E61" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Приложение долго открывается: 6 секунд до главного экрана. Особенно заметно утром.</v>
+      </c>
+      <c r="B62" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C62" t="str">
+        <v>2026-01-10</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 29 часов.</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C63" t="str">
+        <v>2026-01-09</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C64" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="D64">
+        <v>4</v>
+      </c>
+      <c r="E64" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C65" t="str">
+        <v>2026-01-07</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="E65" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Регистрация слишком сложная: 5 шагов — хочется меньше.</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C66" t="str">
+        <v>2026-01-06</v>
+      </c>
+      <c r="D66">
+        <v>2</v>
+      </c>
+      <c r="E66" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B67" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C67" t="str">
+        <v>2026-01-05</v>
+      </c>
+      <c r="D67">
+        <v>2</v>
+      </c>
+      <c r="E67" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C68" t="str">
+        <v>2026-01-04</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C69" t="str">
+        <v>2026-01-03</v>
+      </c>
+      <c r="D69">
+        <v>3</v>
+      </c>
+      <c r="E69" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C70" t="str">
+        <v>2026-01-02</v>
+      </c>
+      <c r="D70">
+        <v>4</v>
+      </c>
+      <c r="E70" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C71" t="str">
+        <v>2026-01-01</v>
+      </c>
+      <c r="D71">
+        <v>2</v>
+      </c>
+      <c r="E71" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Приложение долго открывается: 16 секунд до главного экрана.</v>
+      </c>
+      <c r="B72" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C72" t="str">
+        <v>2025-12-31</v>
+      </c>
+      <c r="D72">
+        <v>2</v>
+      </c>
+      <c r="E72" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 39 часов.</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C73" t="str">
+        <v>2025-12-30</v>
+      </c>
+      <c r="D73">
+        <v>2</v>
+      </c>
+      <c r="E73" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Интерфейс перегружен: Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C74" t="str">
+        <v>2025-12-29</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
+      </c>
+      <c r="E74" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C75" t="str">
+        <v>2025-12-28</v>
+      </c>
+      <c r="D75">
+        <v>2</v>
+      </c>
+      <c r="E75" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Регистрация слишком сложная: 8 шагов — хочется меньше.</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C76" t="str">
+        <v>2025-12-27</v>
+      </c>
+      <c r="D76">
+        <v>3</v>
+      </c>
+      <c r="E76" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B77" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C77" t="str">
+        <v>2025-12-26</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="E77" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C78" t="str">
+        <v>2025-12-25</v>
+      </c>
+      <c r="D78">
+        <v>2</v>
+      </c>
+      <c r="E78" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C79" t="str">
+        <v>2025-12-24</v>
+      </c>
+      <c r="D79">
+        <v>4</v>
+      </c>
+      <c r="E79" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C80" t="str">
+        <v>2025-12-23</v>
+      </c>
+      <c r="D80">
+        <v>2</v>
+      </c>
+      <c r="E80" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C81" t="str">
+        <v>2025-12-22</v>
+      </c>
+      <c r="D81">
+        <v>3</v>
+      </c>
+      <c r="E81" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Приложение долго открывается: 14 секунд до главного экрана. Особенно заметно утром.</v>
+      </c>
+      <c r="B82" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C82" t="str">
+        <v>2025-12-21</v>
+      </c>
+      <c r="D82">
+        <v>3</v>
+      </c>
+      <c r="E82" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 9 часов.</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C83" t="str">
+        <v>2025-12-20</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C84" t="str">
+        <v>2025-12-19</v>
+      </c>
+      <c r="D84">
+        <v>3</v>
+      </c>
+      <c r="E84" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C85" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="D85">
+        <v>3</v>
+      </c>
+      <c r="E85" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Регистрация слишком сложная: 4 шагов — хочется меньше.</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C86" t="str">
+        <v>2025-12-17</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B87" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C87" t="str">
+        <v>2025-12-16</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C88" t="str">
+        <v>2025-12-15</v>
+      </c>
+      <c r="D88">
+        <v>3</v>
+      </c>
+      <c r="E88" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C89" t="str">
+        <v>2025-12-14</v>
+      </c>
+      <c r="D89">
+        <v>2</v>
+      </c>
+      <c r="E89" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C90" t="str">
+        <v>2025-12-13</v>
+      </c>
+      <c r="D90">
+        <v>3</v>
+      </c>
+      <c r="E90" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C91" t="str">
+        <v>2025-12-12</v>
+      </c>
+      <c r="D91">
+        <v>4</v>
+      </c>
+      <c r="E91" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Приложение долго открывается: 12 секунд до главного экрана.</v>
+      </c>
+      <c r="B92" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C92" t="str">
+        <v>2025-12-11</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 19 часов.</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C93" t="str">
+        <v>2025-12-10</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C94" t="str">
+        <v>2025-12-09</v>
+      </c>
+      <c r="D94">
+        <v>4</v>
+      </c>
+      <c r="E94" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C95" t="str">
+        <v>2025-12-08</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Регистрация слишком сложная: 7 шагов — хочется меньше.</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C96" t="str">
+        <v>2025-12-07</v>
+      </c>
+      <c r="D96">
+        <v>2</v>
+      </c>
+      <c r="E96" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B97" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C97" t="str">
+        <v>2025-12-06</v>
+      </c>
+      <c r="D97">
+        <v>2</v>
+      </c>
+      <c r="E97" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C98" t="str">
+        <v>2025-12-05</v>
+      </c>
+      <c r="D98">
+        <v>1</v>
+      </c>
+      <c r="E98" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C99" t="str">
+        <v>2025-12-04</v>
+      </c>
+      <c r="D99">
+        <v>3</v>
+      </c>
+      <c r="E99" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C100" t="str">
+        <v>2025-12-03</v>
+      </c>
+      <c r="D100">
+        <v>4</v>
+      </c>
+      <c r="E100" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C101" t="str">
+        <v>2025-12-02</v>
+      </c>
+      <c r="D101">
+        <v>2</v>
+      </c>
+      <c r="E101" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Приложение долго открывается: 10 секунд до главного экрана. Особенно заметно утром.</v>
+      </c>
+      <c r="B102" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C102" t="str">
+        <v>2025-12-01</v>
+      </c>
+      <c r="D102">
+        <v>2</v>
+      </c>
+      <c r="E102" t="str">
+        <v>performance</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Поддержка отвечает слишком долго — ждал(а) 29 часов.</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C103" t="str">
+        <v>2025-11-30</v>
+      </c>
+      <c r="D103">
+        <v>2</v>
+      </c>
+      <c r="E103" t="str">
+        <v>support</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Интерфейс перегружен: Неочевидная навигация: не могу найти «историю операций».</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C104" t="str">
+        <v>2025-11-29</v>
+      </c>
+      <c r="D104">
+        <v>2</v>
+      </c>
+      <c r="E104" t="str">
+        <v>ux</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>После обновления приложение тормозит и иногда зависает на экране «настройки профиля».</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C105" t="str">
+        <v>2025-11-28</v>
+      </c>
+      <c r="D105">
+        <v>2</v>
+      </c>
+      <c r="E105" t="str">
+        <v>bug</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Регистрация слишком сложная: 10 шагов — хочется меньше.</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C106" t="str">
+        <v>2025-11-27</v>
+      </c>
+      <c r="D106">
+        <v>3</v>
+      </c>
+      <c r="E106" t="str">
+        <v>onboarding</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Оплата не прошла, но деньги списались. Нужен быстрый возврат.</v>
+      </c>
+      <c r="B107" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C107" t="str">
+        <v>2025-11-26</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
+      </c>
+      <c r="E107" t="str">
+        <v>billing</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Показывает ошибку «что-то пошло не так» без объяснения, непонятно что делать.</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Google Play</v>
+      </c>
+      <c r="C108" t="str">
+        <v>2025-11-25</v>
+      </c>
+      <c r="D108">
+        <v>2</v>
+      </c>
+      <c r="E108" t="str">
+        <v>errors</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Пуш-уведомления приходят с задержкой или не приходят вообще.</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Support</v>
+      </c>
+      <c r="C109" t="str">
+        <v>2025-11-24</v>
+      </c>
+      <c r="D109">
+        <v>4</v>
+      </c>
+      <c r="E109" t="str">
+        <v>retention</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Нужен экспорт данных/отчёта — не вижу такой функции.</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C110" t="str">
+        <v>2025-11-23</v>
+      </c>
+      <c r="D110">
+        <v>2</v>
+      </c>
+      <c r="E110" t="str">
+        <v>feature</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Сложно понять, как начать пользоваться: нет подсказок на первом экране.</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Form</v>
+      </c>
+      <c r="C111" t="str">
+        <v>2025-11-22</v>
+      </c>
+      <c r="D111">
+        <v>3</v>
+      </c>
+      <c r="E111" t="str">
+        <v>activation</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Приложение долго открывается: 8 секунд до главного экрана.</v>
+      </c>
+      <c r="B112" t="str">
+        <v>App Store</v>
+      </c>
+      <c r="C112" t="str">
+        <v>2025-11-21</v>
+      </c>
+      <c r="D112">
+        <v>3</v>
+      </c>
+      <c r="E112" t="str">
+        <v>performance</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E112"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A24"/>
   <cols>
-    <col min="1" max="1" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>FeedFocus — пример файла для загрузки отзывов</v>
+        <v>FeedFocus — пример файла для загрузки отзывов (111 строк)</v>
       </c>
     </row>
     <row r="2">
@@ -620,62 +2337,117 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Как тестировать:</v>
+        <v>Что внутри:</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>1) На главной странице выберите «Загрузить CSV / Excel».</v>
+        <v>- Лист «Отзывы»: 111 строк отзывов + дополнительные колонки (source/created_at/rating/tag).</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2) Загрузите этот файл .xlsx.</v>
+        <v>- Лист «Как пользоваться»: инструкция для теста.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3) В выпадающем списке «Колонка с текстом» выберите: text</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>4) Убедитесь, что найдено N отзывов.</v>
+        <v>Как тестировать в FeedFocus:</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>5) Нажмите «Анализировать».</v>
+        <v>1) Откройте сайт FeedFocus.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>2) Выберите режим «Загрузить CSV / Excel».</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Примечание:</v>
+        <v>3) Загрузите этот файл .xlsx.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>- В таблице может быть несколько колонок; FeedFocus берет тексты из выбранной колонки.</v>
+        <v>4) В выпадающем списке «Колонка с текстом» выберите: text</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>- Пустые строки игнорируются.</v>
+        <v>5) Убедитесь, что «Найдено отзывов» = 111 (или меньше, если стоит лимит).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>- Лимит: до 200 отзывов за один анализ.</v>
+        <v>6) Нажмите «Анализировать».</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Что проверять:</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>- Pain points не дублируются и агрегируют похожие формулировки.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>- Появился блок «Главный инсайт».</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>- Страница «Продуктовые гипотезы» открывается.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>- Кнопка «Скачать отчет» скачивает PDF.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Примечания:</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>- FeedFocus берёт тексты из выбранной колонки.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>- Пустые строки должны игнорироваться.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>- Лимит на анализ: до 200 отзывов (если включён).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>